<commit_message>
Implement refined Phase 2 changes against reconciled models and enums; all 16 tests passing
</commit_message>
<xml_diff>
--- a/backend/data/cohort.xlsx
+++ b/backend/data/cohort.xlsx
@@ -2839,7 +2839,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-03T10:39:57.998175</t>
+          <t>2026-08-03T11:05:32.422653</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998187</t>
+          <t>2026-08-06T11:05:32.422668</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998191</t>
+          <t>2026-08-06T11:05:32.422674</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998194</t>
+          <t>2026-08-06T11:05:32.422679</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998196</t>
+          <t>2026-08-06T11:05:32.422683</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998198</t>
+          <t>2026-08-06T11:05:32.422690</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998200</t>
+          <t>2026-08-06T11:05:32.422693</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998204</t>
+          <t>2026-08-06T11:05:32.422697</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998206</t>
+          <t>2026-08-06T11:05:32.422700</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998208</t>
+          <t>2026-08-06T11:05:32.422704</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998210</t>
+          <t>2026-08-06T11:05:32.422707</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998212</t>
+          <t>2026-08-06T11:05:32.422710</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998214</t>
+          <t>2026-08-06T11:05:32.422714</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998216</t>
+          <t>2026-08-06T11:05:32.422717</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998232</t>
+          <t>2026-08-06T11:05:32.422733</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998235</t>
+          <t>2026-08-06T11:05:32.422736</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998237</t>
+          <t>2026-08-06T11:05:32.422739</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998239</t>
+          <t>2026-08-06T11:05:32.422743</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998241</t>
+          <t>2026-08-06T11:05:32.422746</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998243</t>
+          <t>2026-08-06T11:05:32.422749</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-08-06T10:39:57.998245</t>
+          <t>2026-08-06T11:05:32.422753</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-12T10:39:57.998522</t>
+          <t>2026-07-12T11:05:32.423408</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998527</t>
+          <t>2026-07-17T11:05:32.423424</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998532</t>
+          <t>2026-07-17T11:05:32.423432</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998533</t>
+          <t>2026-07-24T11:05:32.423435</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998537</t>
+          <t>2026-07-17T11:05:32.423440</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998539</t>
+          <t>2026-07-24T11:05:32.423444</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998542</t>
+          <t>2026-07-17T11:05:32.423448</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998543</t>
+          <t>2026-07-24T11:05:32.423451</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998545</t>
+          <t>2026-07-17T11:05:32.423455</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998547</t>
+          <t>2026-07-24T11:05:32.423458</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998549</t>
+          <t>2026-07-17T11:05:32.423462</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998551</t>
+          <t>2026-07-24T11:05:32.423465</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998553</t>
+          <t>2026-07-17T11:05:32.423468</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998555</t>
+          <t>2026-07-24T11:05:32.423471</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998557</t>
+          <t>2026-07-17T11:05:32.423475</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998558</t>
+          <t>2026-07-24T11:05:32.423477</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998560</t>
+          <t>2026-07-17T11:05:32.423481</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998562</t>
+          <t>2026-07-24T11:05:32.423484</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998565</t>
+          <t>2026-07-17T11:05:32.423490</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998567</t>
+          <t>2026-07-24T11:05:32.423493</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998569</t>
+          <t>2026-07-17T11:05:32.423496</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998571</t>
+          <t>2026-07-24T11:05:32.423501</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998573</t>
+          <t>2026-07-17T11:05:32.423504</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998575</t>
+          <t>2026-07-24T11:05:32.423507</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998578</t>
+          <t>2026-07-17T11:05:32.423510</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998579</t>
+          <t>2026-07-24T11:05:32.423513</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998581</t>
+          <t>2026-07-17T11:05:32.423517</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998583</t>
+          <t>2026-07-24T11:05:32.423520</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998585</t>
+          <t>2026-07-17T11:05:32.423523</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3821,7 +3821,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998587</t>
+          <t>2026-07-24T11:05:32.423526</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998589</t>
+          <t>2026-07-17T11:05:32.423529</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998590</t>
+          <t>2026-07-24T11:05:32.423532</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998592</t>
+          <t>2026-07-17T11:05:32.423535</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998594</t>
+          <t>2026-07-24T11:05:32.423538</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998596</t>
+          <t>2026-07-17T11:05:32.423542</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998597</t>
+          <t>2026-07-24T11:05:32.423545</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998599</t>
+          <t>2026-07-17T11:05:32.423548</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998601</t>
+          <t>2026-07-24T11:05:32.423551</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998613</t>
+          <t>2026-07-17T11:05:32.423556</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998615</t>
+          <t>2026-07-24T11:05:32.423560</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-07-17T10:39:57.998617</t>
+          <t>2026-07-17T11:05:32.423565</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-24T10:39:57.998618</t>
+          <t>2026-07-24T11:05:32.423573</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 (Corrected) - Update risk banding thresholds, add boundary and hand-reasoned golden tests, update generate_cohort, and fix retain timezone bug
</commit_message>
<xml_diff>
--- a/backend/data/cohort.xlsx
+++ b/backend/data/cohort.xlsx
@@ -513,26 +513,26 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6.15</v>
+        <v>6.1</v>
       </c>
       <c r="D3" t="n">
         <v>0.72</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python</t>
         </is>
       </c>
     </row>
@@ -548,26 +548,26 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python</t>
         </is>
       </c>
     </row>
@@ -583,26 +583,26 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6.45</v>
+        <v>6.1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python</t>
         </is>
       </c>
     </row>
@@ -618,26 +618,26 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python</t>
         </is>
       </c>
     </row>
@@ -653,26 +653,26 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6.75</v>
+        <v>7.2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git</t>
         </is>
       </c>
     </row>
@@ -688,22 +688,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="D8" t="n">
         <v>0.82</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -723,26 +723,26 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7.05</v>
+        <v>7.2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git</t>
         </is>
       </c>
     </row>
@@ -761,19 +761,19 @@
         <v>7.2</v>
       </c>
       <c r="D10" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G10" t="n">
         <v>8</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -793,26 +793,26 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7.35</v>
+        <v>7.2</v>
       </c>
       <c r="D11" t="n">
-        <v>0.88</v>
+        <v>0.82</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git</t>
         </is>
       </c>
     </row>
@@ -828,26 +828,26 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -863,26 +863,26 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7.65</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>5</v>
       </c>
-      <c r="F13" t="n">
-        <v>11</v>
-      </c>
-      <c r="G13" t="n">
-        <v>11</v>
-      </c>
-      <c r="H13" t="n">
-        <v>3</v>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -910,14 +910,14 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -933,26 +933,26 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7.95</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>5</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -968,26 +968,26 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1003,26 +1003,26 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>8.25</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>0.72</v>
+        <v>0.95</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1038,26 +1038,26 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>0.74</v>
+        <v>0.95</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1073,26 +1073,26 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>8.550000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>0.76</v>
+        <v>0.95</v>
       </c>
       <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
         <v>5</v>
       </c>
-      <c r="F19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G19" t="n">
-        <v>17</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1108,26 +1108,26 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>0.78</v>
+        <v>0.95</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1143,26 +1143,26 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8.85</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D21" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>sql,java</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1178,26 +1178,26 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D22" t="n">
-        <v>0.82</v>
+        <v>0.95</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>python,git</t>
+          <t>python,git,sql</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1360,7 +1360,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9">
@@ -1378,7 +1378,7 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
@@ -1389,14 +1389,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
@@ -1411,46 +1411,46 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>STU1002</t>
+          <t>STU1001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>72</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>STU1002</t>
+          <t>STU1001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>74</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14">
@@ -1461,14 +1461,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15">
@@ -1479,20 +1479,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>STU1003</t>
+          <t>STU1002</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1501,34 +1501,34 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>73</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>STU1003</t>
+          <t>STU1002</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>STU1003</t>
+          <t>STU1002</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1537,16 +1537,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>STU1003</t>
+          <t>STU1002</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1555,16 +1555,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>68</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>STU1004</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1576,13 +1576,13 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>STU1004</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1594,31 +1594,31 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>STU1004</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>64</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>STU1004</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1627,57 +1627,57 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>STU1005</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>STU1005</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>77</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>STU1005</t>
+          <t>STU1004</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1690,25 +1690,25 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>STU1005</t>
+          <t>STU1004</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>STU1006</t>
+          <t>STU1004</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1717,34 +1717,34 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>76</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>STU1006</t>
+          <t>STU1004</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>STU1006</t>
+          <t>STU1004</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1753,16 +1753,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>STU1006</t>
+          <t>STU1004</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1771,16 +1771,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>STU1007</t>
+          <t>STU1005</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1792,13 +1792,13 @@
         <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>STU1007</t>
+          <t>STU1005</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1810,31 +1810,31 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>STU1007</t>
+          <t>STU1005</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>STU1007</t>
+          <t>STU1005</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
         <v>72</v>
@@ -1852,79 +1852,79 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>STU1008</t>
+          <t>STU1005</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>STU1008</t>
+          <t>STU1005</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D37" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>STU1008</t>
+          <t>STU1006</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>STU1008</t>
+          <t>STU1006</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>STU1009</t>
+          <t>STU1006</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1933,34 +1933,34 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>STU1009</t>
+          <t>STU1006</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>STU1009</t>
+          <t>STU1006</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1969,16 +1969,16 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>STU1009</t>
+          <t>STU1006</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1987,16 +1987,16 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>STU1010</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2008,13 +2008,13 @@
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>STU1010</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2026,31 +2026,31 @@
         <v>2</v>
       </c>
       <c r="D45" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>STU1010</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>STU1010</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2059,88 +2059,88 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>STU1011</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>STU1011</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>STU1011</t>
+          <t>STU1008</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>STU1011</t>
+          <t>STU1008</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C51" t="n">
         <v>2</v>
       </c>
       <c r="D51" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>STU1012</t>
+          <t>STU1008</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2149,34 +2149,34 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>STU1012</t>
+          <t>STU1008</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>STU1012</t>
+          <t>STU1008</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2185,16 +2185,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>STU1012</t>
+          <t>STU1008</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2203,16 +2203,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>STU1013</t>
+          <t>STU1009</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2224,13 +2224,13 @@
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>STU1013</t>
+          <t>STU1009</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2242,31 +2242,31 @@
         <v>2</v>
       </c>
       <c r="D57" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>STU1013</t>
+          <t>STU1009</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>STU1013</t>
+          <t>STU1009</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2275,88 +2275,88 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>STU1014</t>
+          <t>STU1009</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>STU1014</t>
+          <t>STU1009</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>86</v>
+        <v>70</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>STU1014</t>
+          <t>STU1010</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>74</v>
+        <v>85</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>STU1014</t>
+          <t>STU1010</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>2</v>
       </c>
       <c r="D63" t="n">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>STU1015</t>
+          <t>STU1010</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2365,34 +2365,34 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>STU1015</t>
+          <t>STU1010</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>STU1015</t>
+          <t>STU1010</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2401,16 +2401,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D66" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>STU1015</t>
+          <t>STU1010</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2419,16 +2419,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D67" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>STU1016</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2440,13 +2440,13 @@
         <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>STU1016</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2464,25 +2464,25 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>STU1016</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D70" t="n">
-        <v>76</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>STU1016</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2491,88 +2491,88 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>STU1017</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D72" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>STU1017</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>STU1017</t>
+          <t>STU1012</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>STU1017</t>
+          <t>STU1012</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C75" t="n">
         <v>2</v>
       </c>
       <c r="D75" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>STU1018</t>
+          <t>STU1012</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2581,34 +2581,34 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>STU1018</t>
+          <t>STU1012</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>STU1018</t>
+          <t>STU1012</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2617,16 +2617,16 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D78" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>STU1018</t>
+          <t>STU1012</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2635,16 +2635,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>STU1019</t>
+          <t>STU1013</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2656,13 +2656,13 @@
         <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>STU1019</t>
+          <t>STU1013</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2674,31 +2674,31 @@
         <v>2</v>
       </c>
       <c r="D81" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>STU1019</t>
+          <t>STU1013</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>STU1019</t>
+          <t>STU1013</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2707,82 +2707,802 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D83" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>STU1020</t>
+          <t>STU1013</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>STU1020</t>
+          <t>STU1013</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>STU1020</t>
+          <t>STU1014</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C86" t="n">
         <v>1</v>
       </c>
       <c r="D86" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>STU1014</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>STU1014</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>3</v>
+      </c>
+      <c r="D88" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>STU1014</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>STU1014</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>STU1014</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>3</v>
+      </c>
+      <c r="D91" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>STU1015</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>STU1015</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>STU1015</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>3</v>
+      </c>
+      <c r="D94" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>STU1015</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>STU1015</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>STU1015</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>3</v>
+      </c>
+      <c r="D97" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>STU1016</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>STU1016</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>STU1016</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>3</v>
+      </c>
+      <c r="D100" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>STU1016</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>STU1016</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>2</v>
+      </c>
+      <c r="D102" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>STU1016</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>3</v>
+      </c>
+      <c r="D103" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>STU1017</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>STU1017</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>2</v>
+      </c>
+      <c r="D105" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>STU1017</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>3</v>
+      </c>
+      <c r="D106" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>STU1017</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>STU1017</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>2</v>
+      </c>
+      <c r="D108" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>STU1017</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>3</v>
+      </c>
+      <c r="D109" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>STU1018</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>STU1018</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>2</v>
+      </c>
+      <c r="D111" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>STU1018</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>3</v>
+      </c>
+      <c r="D112" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>STU1018</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>STU1018</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>2</v>
+      </c>
+      <c r="D114" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>STU1018</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>3</v>
+      </c>
+      <c r="D115" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>STU1019</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>STU1019</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>2</v>
+      </c>
+      <c r="D117" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>STU1019</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>3</v>
+      </c>
+      <c r="D118" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>STU1019</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
+      </c>
+      <c r="D119" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>STU1019</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>2</v>
+      </c>
+      <c r="D120" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>STU1019</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>3</v>
+      </c>
+      <c r="D121" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
           <t>STU1020</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
-      <c r="C87" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" t="n">
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="n">
         <v>85</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>STU1020</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>2</v>
+      </c>
+      <c r="D123" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>STU1020</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>3</v>
+      </c>
+      <c r="D124" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>STU1020</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>STU1020</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>2</v>
+      </c>
+      <c r="D126" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>STU1020</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D127" t="n">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2839,7 +3559,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-03T11:05:32.422653</t>
+          <t>2026-08-03T17:14:01.108167</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -2862,14 +3582,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422668</t>
+          <t>2026-07-27T17:14:01.108178</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4">
@@ -2880,19 +3600,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422674</t>
+          <t>2026-07-27T17:14:01.108181</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5">
@@ -2908,14 +3628,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422679</t>
+          <t>2026-07-27T17:14:01.108184</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">
@@ -2926,19 +3646,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422683</t>
+          <t>2026-07-27T17:14:01.108186</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -2954,14 +3674,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422690</t>
+          <t>2026-08-01T17:14:01.108188</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="8">
@@ -2972,19 +3692,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422693</t>
+          <t>2026-08-01T17:14:01.108192</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="9">
@@ -3000,14 +3720,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422697</t>
+          <t>2026-08-01T17:14:01.108195</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="10">
@@ -3018,19 +3738,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422700</t>
+          <t>2026-08-01T17:14:01.108197</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="11">
@@ -3046,14 +3766,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422704</t>
+          <t>2026-08-01T17:14:01.108199</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="12">
@@ -3064,19 +3784,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422707</t>
+          <t>2026-08-11T17:14:01.108201</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="13">
@@ -3092,14 +3812,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422710</t>
+          <t>2026-08-11T17:14:01.108203</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E13" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="14">
@@ -3110,19 +3830,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422714</t>
+          <t>2026-08-11T17:14:01.108206</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="15">
@@ -3138,14 +3858,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422717</t>
+          <t>2026-08-11T17:14:01.108208</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="16">
@@ -3156,19 +3876,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422733</t>
+          <t>2026-08-11T17:14:01.108210</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="17">
@@ -3184,14 +3904,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422736</t>
+          <t>2026-08-11T17:14:01.108212</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="18">
@@ -3202,19 +3922,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422739</t>
+          <t>2026-08-11T17:14:01.108213</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="19">
@@ -3230,14 +3950,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422743</t>
+          <t>2026-08-11T17:14:01.108215</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="20">
@@ -3248,19 +3968,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422746</t>
+          <t>2026-08-11T17:14:01.108217</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="21">
@@ -3276,14 +3996,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422749</t>
+          <t>2026-08-11T17:14:01.108221</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="22">
@@ -3294,19 +4014,19 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-08-06T11:05:32.422753</t>
+          <t>2026-08-11T17:14:01.108223</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
     </row>
   </sheetData>
@@ -3373,7 +4093,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-12T11:05:32.423408</t>
+          <t>2026-07-12T17:14:01.108458</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -3387,7 +4107,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423424</t>
+          <t>2026-07-17T17:14:01.108463</t>
         </is>
       </c>
     </row>
@@ -3404,7 +4124,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423432</t>
+          <t>2026-07-17T17:14:01.108467</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -3418,7 +4138,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423435</t>
+          <t>2026-07-24T17:14:01.108468</t>
         </is>
       </c>
     </row>
@@ -3435,7 +4155,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423440</t>
+          <t>2026-07-17T17:14:01.108471</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -3449,7 +4169,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423444</t>
+          <t>2026-07-24T17:14:01.108474</t>
         </is>
       </c>
     </row>
@@ -3466,7 +4186,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423448</t>
+          <t>2026-07-17T17:14:01.108476</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -3480,7 +4200,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423451</t>
+          <t>2026-07-24T17:14:01.108478</t>
         </is>
       </c>
     </row>
@@ -3497,7 +4217,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423455</t>
+          <t>2026-07-17T17:14:01.108480</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -3511,7 +4231,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423458</t>
+          <t>2026-07-24T17:14:01.108482</t>
         </is>
       </c>
     </row>
@@ -3528,7 +4248,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423462</t>
+          <t>2026-07-17T17:14:01.108484</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -3542,7 +4262,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423465</t>
+          <t>2026-07-24T17:14:01.108488</t>
         </is>
       </c>
     </row>
@@ -3559,7 +4279,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423468</t>
+          <t>2026-07-17T17:14:01.108490</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -3573,7 +4293,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423471</t>
+          <t>2026-07-24T17:14:01.108491</t>
         </is>
       </c>
     </row>
@@ -3590,7 +4310,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423475</t>
+          <t>2026-07-17T17:14:01.108493</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3604,7 +4324,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423477</t>
+          <t>2026-07-24T17:14:01.108495</t>
         </is>
       </c>
     </row>
@@ -3621,7 +4341,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423481</t>
+          <t>2026-07-17T17:14:01.108497</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3635,7 +4355,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423484</t>
+          <t>2026-07-24T17:14:01.108499</t>
         </is>
       </c>
     </row>
@@ -3652,7 +4372,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423490</t>
+          <t>2026-07-17T17:14:01.108502</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3666,7 +4386,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423493</t>
+          <t>2026-07-24T17:14:01.108504</t>
         </is>
       </c>
     </row>
@@ -3683,7 +4403,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423496</t>
+          <t>2026-07-17T17:14:01.108507</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3697,7 +4417,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423501</t>
+          <t>2026-07-24T17:14:01.108509</t>
         </is>
       </c>
     </row>
@@ -3714,7 +4434,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423504</t>
+          <t>2026-07-17T17:14:01.108511</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3728,7 +4448,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423507</t>
+          <t>2026-07-24T17:14:01.108512</t>
         </is>
       </c>
     </row>
@@ -3745,7 +4465,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423510</t>
+          <t>2026-07-17T17:14:01.108514</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3759,7 +4479,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423513</t>
+          <t>2026-07-24T17:14:01.108516</t>
         </is>
       </c>
     </row>
@@ -3776,7 +4496,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423517</t>
+          <t>2026-07-17T17:14:01.108518</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3790,7 +4510,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423520</t>
+          <t>2026-07-24T17:14:01.108520</t>
         </is>
       </c>
     </row>
@@ -3807,7 +4527,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423523</t>
+          <t>2026-07-17T17:14:01.108522</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3821,7 +4541,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423526</t>
+          <t>2026-07-24T17:14:01.108523</t>
         </is>
       </c>
     </row>
@@ -3838,7 +4558,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423529</t>
+          <t>2026-07-17T17:14:01.108525</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3852,7 +4572,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423532</t>
+          <t>2026-07-24T17:14:01.108527</t>
         </is>
       </c>
     </row>
@@ -3869,7 +4589,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423535</t>
+          <t>2026-07-17T17:14:01.108529</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3883,7 +4603,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423538</t>
+          <t>2026-07-24T17:14:01.108530</t>
         </is>
       </c>
     </row>
@@ -3900,7 +4620,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423542</t>
+          <t>2026-07-17T17:14:01.108532</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -3914,7 +4634,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423545</t>
+          <t>2026-07-24T17:14:01.108534</t>
         </is>
       </c>
     </row>
@@ -3931,7 +4651,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423548</t>
+          <t>2026-07-17T17:14:01.108536</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -3945,7 +4665,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423551</t>
+          <t>2026-07-24T17:14:01.108537</t>
         </is>
       </c>
     </row>
@@ -3962,7 +4682,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423556</t>
+          <t>2026-07-17T17:14:01.108539</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -3976,7 +4696,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423560</t>
+          <t>2026-07-24T17:14:01.108541</t>
         </is>
       </c>
     </row>
@@ -3993,7 +4713,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-07-17T11:05:32.423565</t>
+          <t>2026-07-17T17:14:01.108543</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -4007,7 +4727,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-24T11:05:32.423573</t>
+          <t>2026-07-24T17:14:01.108544</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
phase5: demo stabilization lock
- risk.py: calibrated banding 45/25 (High>=45, Medium>=25, else Low)
- SPEC.md: updated banding doc to 45/25; renamed product to Drishta
- language.py: GEMINI_API_KEY; all user-facing strings renamed Polaris->Drishta
  (templated fallbacks, LLM prompts); clean_and_truncate strips drishta label too
- generate_cohort.py: High-risk students now have distinct realistic names
  (Rohan Mehta, Priya Sharma, Arjun Nair, Fatima Khan) with varied inputs
  and distinct declining score profiles so dashboard scores differ (71/64/76/59)
- cohort.xlsx: regenerated with new High-risk profiles
  spread: 4 High / 6 Medium / 11 Low
  Aisha baseline Medium(35) -> natural drift High(47) + flag_at_risk fires
- tests: Drishta Mentor assertions; exams[0].days_to_exam=5 in transition test
  32/32 pass, no hang, 4.4s
</commit_message>
<xml_diff>
--- a/backend/data/cohort.xlsx
+++ b/backend/data/cohort.xlsx
@@ -509,23 +509,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Student 1</t>
+          <t>Rohan Mehta</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.72</v>
+        <v>0.68</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G3" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -544,14 +544,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Student 2</t>
+          <t>Priya Sharma</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="D4" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="E4" t="n">
         <v>8</v>
@@ -560,14 +560,14 @@
         <v>12</v>
       </c>
       <c r="G4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>java</t>
         </is>
       </c>
     </row>
@@ -579,30 +579,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Student 3</t>
+          <t>Arjun Nair</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>c++</t>
         </is>
       </c>
     </row>
@@ -614,30 +614,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Student 4</t>
+          <t>Fatima Khan</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="D6" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>python,sql</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9">
@@ -1378,7 +1378,7 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -1396,7 +1396,7 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -1414,7 +1414,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12">
@@ -1450,7 +1450,7 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14">
@@ -1486,7 +1486,7 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16">
@@ -1504,7 +1504,7 @@
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -1540,7 +1540,7 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19">
@@ -1558,7 +1558,7 @@
         <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20">
@@ -1576,7 +1576,7 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21">
@@ -1594,7 +1594,7 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22">
@@ -1612,7 +1612,7 @@
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23">
@@ -1630,7 +1630,7 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24">
@@ -1648,7 +1648,7 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25">
@@ -1666,7 +1666,7 @@
         <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26">
@@ -1684,7 +1684,7 @@
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27">
@@ -1702,7 +1702,7 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28">
@@ -1720,7 +1720,7 @@
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29">
@@ -1738,7 +1738,7 @@
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30">
@@ -1756,7 +1756,7 @@
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31">
@@ -1774,7 +1774,7 @@
         <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-03T17:14:01.108167</t>
+          <t>2026-08-03T22:05:40.061456</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -3582,14 +3582,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-27T17:14:01.108178</t>
+          <t>2026-07-26T22:05:40.061478</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="4">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-27T17:14:01.108181</t>
+          <t>2026-07-28T22:05:40.061484</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
         <v>0.2</v>
@@ -3628,14 +3628,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-27T17:14:01.108184</t>
+          <t>2026-07-25T22:05:40.061489</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6">
@@ -3651,14 +3651,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-27T17:14:01.108186</t>
+          <t>2026-07-27T22:05:40.061493</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="7">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-01T17:14:01.108188</t>
+          <t>2026-08-01T22:05:40.061500</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-01T17:14:01.108192</t>
+          <t>2026-08-01T22:05:40.061509</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-01T17:14:01.108195</t>
+          <t>2026-08-01T22:05:40.061513</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-01T17:14:01.108197</t>
+          <t>2026-08-01T22:05:40.061517</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-01T17:14:01.108199</t>
+          <t>2026-08-01T22:05:40.061521</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108201</t>
+          <t>2026-08-11T22:05:40.061525</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108203</t>
+          <t>2026-08-11T22:05:40.061529</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108206</t>
+          <t>2026-08-11T22:05:40.061552</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108208</t>
+          <t>2026-08-11T22:05:40.061556</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108210</t>
+          <t>2026-08-11T22:05:40.061559</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108212</t>
+          <t>2026-08-11T22:05:40.061563</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108213</t>
+          <t>2026-08-11T22:05:40.061567</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108215</t>
+          <t>2026-08-11T22:05:40.061570</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108217</t>
+          <t>2026-08-11T22:05:40.061574</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108221</t>
+          <t>2026-08-11T22:05:40.061577</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-08-11T17:14:01.108223</t>
+          <t>2026-08-11T22:05:40.061581</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-12T17:14:01.108458</t>
+          <t>2026-07-12T22:05:40.062145</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108463</t>
+          <t>2026-07-17T22:05:40.062156</t>
         </is>
       </c>
     </row>
@@ -4119,12 +4119,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108467</t>
+          <t>2026-07-17T22:05:40.062163</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108468</t>
+          <t>2026-07-24T22:05:40.062166</t>
         </is>
       </c>
     </row>
@@ -4150,12 +4150,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108471</t>
+          <t>2026-07-17T22:05:40.062172</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -4169,7 +4169,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108474</t>
+          <t>2026-07-24T22:05:40.062175</t>
         </is>
       </c>
     </row>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108476</t>
+          <t>2026-07-17T22:05:40.062179</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108478</t>
+          <t>2026-07-24T22:05:40.062182</t>
         </is>
       </c>
     </row>
@@ -4212,12 +4212,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108480</t>
+          <t>2026-07-17T22:05:40.062186</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108482</t>
+          <t>2026-07-24T22:05:40.062188</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108484</t>
+          <t>2026-07-17T22:05:40.062195</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108488</t>
+          <t>2026-07-24T22:05:40.062198</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108490</t>
+          <t>2026-07-17T22:05:40.062202</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108491</t>
+          <t>2026-07-24T22:05:40.062205</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108493</t>
+          <t>2026-07-17T22:05:40.062209</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108495</t>
+          <t>2026-07-24T22:05:40.062212</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108497</t>
+          <t>2026-07-17T22:05:40.062217</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108499</t>
+          <t>2026-07-24T22:05:40.062219</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108502</t>
+          <t>2026-07-17T22:05:40.062225</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108504</t>
+          <t>2026-07-24T22:05:40.062228</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108507</t>
+          <t>2026-07-17T22:05:40.062232</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108509</t>
+          <t>2026-07-24T22:05:40.062235</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108511</t>
+          <t>2026-07-17T22:05:40.062239</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108512</t>
+          <t>2026-07-24T22:05:40.062241</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108514</t>
+          <t>2026-07-17T22:05:40.062245</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108516</t>
+          <t>2026-07-24T22:05:40.062248</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108518</t>
+          <t>2026-07-17T22:05:40.062251</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108520</t>
+          <t>2026-07-24T22:05:40.062254</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108522</t>
+          <t>2026-07-17T22:05:40.062257</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108523</t>
+          <t>2026-07-24T22:05:40.062260</t>
         </is>
       </c>
     </row>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108525</t>
+          <t>2026-07-17T22:05:40.062263</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108527</t>
+          <t>2026-07-24T22:05:40.062266</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108529</t>
+          <t>2026-07-17T22:05:40.062270</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108530</t>
+          <t>2026-07-24T22:05:40.062273</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108532</t>
+          <t>2026-07-17T22:05:40.062277</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108534</t>
+          <t>2026-07-24T22:05:40.062280</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108536</t>
+          <t>2026-07-17T22:05:40.062283</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108537</t>
+          <t>2026-07-24T22:05:40.062286</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108539</t>
+          <t>2026-07-17T22:05:40.062289</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108541</t>
+          <t>2026-07-24T22:05:40.062292</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-07-17T17:14:01.108543</t>
+          <t>2026-07-17T22:05:40.062295</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-24T17:14:01.108544</t>
+          <t>2026-07-24T22:05:40.062298</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: integrate real backend end-to-end and fix E2E tests
</commit_message>
<xml_diff>
--- a/backend/data/cohort.xlsx
+++ b/backend/data/cohort.xlsx
@@ -3589,7 +3589,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-03T23:00:45.091325</t>
+          <t>2026-08-04T05:31:06.039956</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-26T23:00:45.091342</t>
+          <t>2026-07-27T05:31:06.039970</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-28T23:00:45.091348</t>
+          <t>2026-07-29T05:31:06.039976</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-25T23:00:45.091353</t>
+          <t>2026-07-26T05:31:06.039978</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-27T23:00:45.091357</t>
+          <t>2026-07-28T05:31:06.039980</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-01T23:00:45.091388</t>
+          <t>2026-08-02T05:31:06.039985</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -3727,7 +3727,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-01T23:00:45.091394</t>
+          <t>2026-08-02T05:31:06.039988</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-01T23:00:45.091399</t>
+          <t>2026-08-02T05:31:06.039990</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-01T23:00:45.091403</t>
+          <t>2026-08-02T05:31:06.039992</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-01T23:00:45.091407</t>
+          <t>2026-08-02T05:31:06.039995</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091411</t>
+          <t>2026-08-12T05:31:06.039997</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091415</t>
+          <t>2026-08-12T05:31:06.040000</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091420</t>
+          <t>2026-08-12T05:31:06.040002</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091423</t>
+          <t>2026-08-12T05:31:06.040004</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091427</t>
+          <t>2026-08-12T05:31:06.040006</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091431</t>
+          <t>2026-08-12T05:31:06.040008</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091434</t>
+          <t>2026-08-12T05:31:06.040010</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091438</t>
+          <t>2026-08-12T05:31:06.040012</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091442</t>
+          <t>2026-08-12T05:31:06.040014</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091445</t>
+          <t>2026-08-12T05:31:06.040016</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-08-11T23:00:45.091449</t>
+          <t>2026-08-12T05:31:06.040018</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-12T23:00:45.091956</t>
+          <t>2026-07-13T05:31:06.040395</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.091966</t>
+          <t>2026-07-18T05:31:06.040405</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4154,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.091974</t>
+          <t>2026-07-18T05:31:06.040409</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.091977</t>
+          <t>2026-07-25T05:31:06.040411</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.091983</t>
+          <t>2026-07-18T05:31:06.040414</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.091987</t>
+          <t>2026-07-25T05:31:06.040417</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.091992</t>
+          <t>2026-07-18T05:31:06.040419</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.091995</t>
+          <t>2026-07-25T05:31:06.040421</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.091999</t>
+          <t>2026-07-18T05:31:06.040425</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092002</t>
+          <t>2026-07-25T05:31:06.040426</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092009</t>
+          <t>2026-07-18T05:31:06.040431</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092012</t>
+          <t>2026-07-25T05:31:06.040433</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092017</t>
+          <t>2026-07-18T05:31:06.040435</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -4323,7 +4323,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092021</t>
+          <t>2026-07-25T05:31:06.040437</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4340,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092025</t>
+          <t>2026-07-18T05:31:06.040440</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092029</t>
+          <t>2026-07-25T05:31:06.040441</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092033</t>
+          <t>2026-07-18T05:31:06.040443</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092036</t>
+          <t>2026-07-25T05:31:06.040445</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092042</t>
+          <t>2026-07-18T05:31:06.040447</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092046</t>
+          <t>2026-07-25T05:31:06.040450</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092050</t>
+          <t>2026-07-18T05:31:06.040452</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092053</t>
+          <t>2026-07-25T05:31:06.040454</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092056</t>
+          <t>2026-07-18T05:31:06.040456</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092060</t>
+          <t>2026-07-25T05:31:06.040458</t>
         </is>
       </c>
     </row>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092063</t>
+          <t>2026-07-18T05:31:06.040460</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092066</t>
+          <t>2026-07-25T05:31:06.040461</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092070</t>
+          <t>2026-07-18T05:31:06.040463</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092073</t>
+          <t>2026-07-25T05:31:06.040466</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092078</t>
+          <t>2026-07-18T05:31:06.040469</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092081</t>
+          <t>2026-07-25T05:31:06.040470</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092084</t>
+          <t>2026-07-18T05:31:06.040472</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092087</t>
+          <t>2026-07-25T05:31:06.040474</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092091</t>
+          <t>2026-07-18T05:31:06.040476</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092095</t>
+          <t>2026-07-25T05:31:06.040478</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4650,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092099</t>
+          <t>2026-07-18T05:31:06.040480</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092102</t>
+          <t>2026-07-25T05:31:06.040482</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092105</t>
+          <t>2026-07-18T05:31:06.040484</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092108</t>
+          <t>2026-07-25T05:31:06.040485</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092112</t>
+          <t>2026-07-18T05:31:06.040487</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092115</t>
+          <t>2026-07-25T05:31:06.040489</t>
         </is>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-07-17T23:00:45.092119</t>
+          <t>2026-07-18T05:31:06.040491</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-24T23:00:45.092122</t>
+          <t>2026-07-25T05:31:06.040493</t>
         </is>
       </c>
     </row>

</xml_diff>